<commit_message>
Temperature, common time range, start of pig exp
Temperature:
- now temperature at a height of 20 cm above the ground instead of 10 bellow is used

Common time range:
- current algoritm did not work on for pig data and was therefore changed

Start of pig exp:
changed to start at 11:40 (actual start) instead of 11:48 (first meassurement)
</commit_message>
<xml_diff>
--- a/Field-trails/2025-10-28-cattle-slurry/DFC overview cattle.xlsx
+++ b/Field-trails/2025-10-28-cattle-slurry/DFC overview cattle.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\Cattle-Slurry 2025-10-28\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\2025-10-28-cattle-slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76B749A9-66EF-470D-A60F-5B8B464E9C09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B918CD5A-03A6-4C98-8444-05775806C3D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -607,7 +607,8 @@
     <col min="6" max="6" width="16.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.88671875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Scripts last lab experiment, continued modelling
</commit_message>
<xml_diff>
--- a/Field-trails/2025-10-28-cattle-slurry/DFC overview cattle.xlsx
+++ b/Field-trails/2025-10-28-cattle-slurry/DFC overview cattle.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\2025-10-28-cattle-slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAAB7481-C114-4C83-8E13-5F0B5714BEFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5951B5F-3F3A-4D57-8C2B-5438BDDEBA5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -283,12 +283,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -303,12 +309,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="20" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -733,20 +742,20 @@
       <c r="D3">
         <v>4</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="6">
         <v>0.44166666666666665</v>
       </c>
-      <c r="H3" s="4">
+      <c r="H3" s="7">
         <f>H2+(8/60)</f>
         <v>0.13333333333333333</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="6">
         <v>0.45694444444444443</v>
       </c>
       <c r="P3">
@@ -795,7 +804,7 @@
         <v>0.22908513701242167</v>
       </c>
       <c r="L4" s="4">
-        <f t="shared" ref="L3:L13" si="1">K4*60</f>
+        <f t="shared" ref="L4:L13" si="1">K4*60</f>
         <v>13.745108220745299</v>
       </c>
     </row>
@@ -809,20 +818,20 @@
       <c r="D5">
         <v>7</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="6">
         <v>0.452777777777778</v>
       </c>
-      <c r="H5" s="4">
+      <c r="H5" s="7">
         <f t="shared" si="0"/>
         <v>0.4</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="6">
         <v>0.468055555555556</v>
       </c>
     </row>
@@ -1025,20 +1034,20 @@
       <c r="D11">
         <v>13</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G11" s="3">
+      <c r="G11" s="6">
         <v>0.48611111111111099</v>
       </c>
-      <c r="H11" s="4">
+      <c r="H11" s="7">
         <f t="shared" si="0"/>
         <v>1.2</v>
       </c>
-      <c r="I11" s="3">
+      <c r="I11" s="6">
         <v>0.50138888888888899</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-modelled cattleFiels as trailing shoe
</commit_message>
<xml_diff>
--- a/Field-trails/2025-10-28-cattle-slurry/DFC overview cattle.xlsx
+++ b/Field-trails/2025-10-28-cattle-slurry/DFC overview cattle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Field-trails\2025-10-28-cattle-slurry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5951B5F-3F3A-4D57-8C2B-5438BDDEBA5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A815C21-3728-4049-9809-887D2C051D7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="32">
   <si>
     <t>Comments</t>
   </si>
@@ -234,6 +234,9 @@
   </si>
   <si>
     <t>AER [1/min]</t>
+  </si>
+  <si>
+    <t>Wi</t>
   </si>
 </sst>
 </file>
@@ -703,8 +706,8 @@
       <c r="H2" s="4">
         <v>0</v>
       </c>
-      <c r="I2" s="3">
-        <v>0.4513888888888889</v>
+      <c r="I2" s="3" t="s">
+        <v>31</v>
       </c>
       <c r="J2">
         <f>(F2^0.5)*$P$2</f>
@@ -718,9 +721,9 @@
         <f>K2*60</f>
         <v>13.745108220745299</v>
       </c>
-      <c r="N2" s="3">
+      <c r="N2" s="3" t="e">
         <f>I2-G2</f>
-        <v>1.5277777777777779E-2</v>
+        <v>#VALUE!</v>
       </c>
       <c r="P2">
         <v>3</v>

</xml_diff>